<commit_message>
16/06/2026 Marketing Excel, precio unitario en lineas OV y flujo ampliado
Incluye envio de Costo/SalesPrice a Dynamics, scripts marketing, CORS y libros Excel de prueba.
</commit_message>
<xml_diff>
--- a/Prueba_Ov.xlsx
+++ b/Prueba_Ov.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\BecarioQR\Alexis\Prueba_Ov\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1D9C0F6A-B30C-4DB6-9DC8-80DCF421CAE5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E22E7A8E-CF6A-4B9B-8067-DD1BAC4DF3F1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" activeTab="2" xr2:uid="{BD67EBF7-4FB8-450E-AC59-1504186C6C63}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" activeTab="3" xr2:uid="{BD67EBF7-4FB8-450E-AC59-1504186C6C63}"/>
   </bookViews>
   <sheets>
     <sheet name="Conexión" sheetId="4" r:id="rId1"/>
@@ -110,19 +110,19 @@
     <t>https://unexpired-joyfully-exfoliate.ngrok-free.dev</t>
   </si>
   <si>
-    <t>ERROR</t>
-  </si>
-  <si>
     <t>Prueba desde excel odata</t>
   </si>
   <si>
     <t>OV0027972</t>
   </si>
   <si>
-    <t>2026-05-25T21:31:00.028Z</t>
-  </si>
-  <si>
-    <t>HTTP 500: {"timestamp":1779744659742,"status":500,"error":"Internal Server Error","message":"Dynamics HTTP 400 en https://olnatura-produccion.operations.dynamics.com/data/D365SalesOrderLines [HTTP 400] {\r\n  \"error\":{\r\n    \"code\":\"\",\"message\":\"An error has occurred.\",\"innererror\":{\r\n      \"message\":\"Write failed for table row of type 'SalesOrderLineD365SalesEntity'. Infolog: Warning: No existe ning\\u00fan registro coincidente con la clave 'DisplayProductNumber': 50000595453 para el origen de datos \\\"EcoResDistinctProduct\\\"..\",\"type\":\"Microsoft.Dynamics.Platform.Integration.Services.OData.AxODataWriteException\",\"stacktrace\":\"   at Microsoft.Dynamics.Platform.Integration.Services.OData.Update.UpdateProcessor.CreateEntity_Save(ChangeOperationContext context, ChangeInfo changeInfo)\\r\\n   at Microsoft.Dynamics.Platform.Integration.Services.OData.Update.ChangeInfo.ExecuteActionsInCompanyContext(IEnumerable`1 actionList, ChangeOperationContext operationContext)\\r\\n   at Microsoft.Dynamics.Platform.Integration.Services.OData.Update.ChangeInfo.TrySave(ChangeOperationContext operationContext)\\r\\n   at Microsoft.Dynamics.Platform.Integration.Services.OData.Update.UpdateManager.SaveChanges()\\r\\n   at Microsoft.Dynamics.Platform.Integration.Services.OData.AxODataDelegatingHandler.&lt;SaveChangesAsync&gt;d__3.MoveNext()\"\r\n    }\r\n  }\r\n}","path":"/api/pedidos/lineas"}</t>
+    <t>CONEXION OK</t>
+  </si>
+  <si>
+    <t>Conexion OK con Dynamics FO y token Azure valido.</t>
+  </si>
+  <si>
+    <t>2026-05-28T21:36:17.457Z</t>
   </si>
 </sst>
 </file>
@@ -215,13 +215,13 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1"/>
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hipervínculo" xfId="1" builtinId="8"/>
@@ -250,6 +250,26 @@
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
+      <numFmt numFmtId="19" formatCode="dd/mm/yyyy"/>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="19" formatCode="dd/mm/yyyy"/>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
       <numFmt numFmtId="1" formatCode="0"/>
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
@@ -271,26 +291,6 @@
     </dxf>
     <dxf>
       <numFmt numFmtId="1" formatCode="0"/>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="19" formatCode="dd/mm/yyyy"/>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="19" formatCode="dd/mm/yyyy"/>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
@@ -562,29 +562,29 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{B4E0EA3F-D5B0-4BF4-B8B4-44E41EA1033B}" name="tblPedido" displayName="tblPedido" ref="A2:E3" totalsRowShown="0" dataDxfId="19">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{B4E0EA3F-D5B0-4BF4-B8B4-44E41EA1033B}" name="tblPedido" displayName="tblPedido" ref="A2:E3" totalsRowShown="0" dataDxfId="12">
   <autoFilter ref="A2:E3" xr:uid="{B4E0EA3F-D5B0-4BF4-B8B4-44E41EA1033B}"/>
   <tableColumns count="5">
-    <tableColumn id="1" xr3:uid="{0C93B2BB-158F-4E9B-BE56-6623ADFF1450}" name="Cliente" dataDxfId="18"/>
-    <tableColumn id="2" xr3:uid="{2322016B-EA9D-4FBD-8053-352416DCCFA6}" name="Referencia de cliente " dataDxfId="17"/>
-    <tableColumn id="3" xr3:uid="{A525BD44-1605-40E7-B2A3-EC7B65736888}" name="Descripción de pedido" dataDxfId="16"/>
-    <tableColumn id="4" xr3:uid="{FAB2371F-423F-4FA2-ABAE-B55B3515917C}" name="Fecha de envio solicitada " dataDxfId="15"/>
-    <tableColumn id="5" xr3:uid="{41FD4E4E-29F4-4C39-94DB-1FAED0ED38C1}" name="Fecha de recepción solicitada " dataDxfId="14"/>
+    <tableColumn id="1" xr3:uid="{0C93B2BB-158F-4E9B-BE56-6623ADFF1450}" name="Cliente" dataDxfId="11"/>
+    <tableColumn id="2" xr3:uid="{2322016B-EA9D-4FBD-8053-352416DCCFA6}" name="Referencia de cliente " dataDxfId="10"/>
+    <tableColumn id="3" xr3:uid="{A525BD44-1605-40E7-B2A3-EC7B65736888}" name="Descripción de pedido" dataDxfId="9"/>
+    <tableColumn id="4" xr3:uid="{FAB2371F-423F-4FA2-ABAE-B55B3515917C}" name="Fecha de envio solicitada " dataDxfId="8"/>
+    <tableColumn id="5" xr3:uid="{41FD4E4E-29F4-4C39-94DB-1FAED0ED38C1}" name="Fecha de recepción solicitada " dataDxfId="7"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{C899FE4B-947F-4751-A623-19690F740D53}" name="tblLineas" displayName="tblLineas" ref="A2:F3" totalsRowShown="0" dataDxfId="13">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{C899FE4B-947F-4751-A623-19690F740D53}" name="tblLineas" displayName="tblLineas" ref="A2:F3" totalsRowShown="0" dataDxfId="19">
   <autoFilter ref="A2:F3" xr:uid="{C899FE4B-947F-4751-A623-19690F740D53}"/>
   <tableColumns count="6">
-    <tableColumn id="1" xr3:uid="{D61D6DC2-B681-4F4F-B494-2F569007F324}" name="Codigo_Articulo" dataDxfId="12"/>
-    <tableColumn id="2" xr3:uid="{48B651B6-1934-4211-9148-EE699069241B}" name="Cantidad" dataDxfId="11"/>
-    <tableColumn id="3" xr3:uid="{00763216-ACDD-418D-9D9B-0F02D296387E}" name="PrecioUnitario" dataDxfId="10"/>
-    <tableColumn id="4" xr3:uid="{6E6D0715-DC12-452D-8B1E-CF365D12A12B}" name="Porcentaje de descuento" dataDxfId="9"/>
-    <tableColumn id="5" xr3:uid="{B38FD930-D30F-48BA-94A4-68837908CE07}" name="Fecha de envio" dataDxfId="8"/>
-    <tableColumn id="6" xr3:uid="{C066523A-73B4-4BFA-9EA4-BBFD947FE4DC}" name="Comentarios" dataDxfId="7"/>
+    <tableColumn id="1" xr3:uid="{D61D6DC2-B681-4F4F-B494-2F569007F324}" name="Codigo_Articulo" dataDxfId="18"/>
+    <tableColumn id="2" xr3:uid="{48B651B6-1934-4211-9148-EE699069241B}" name="Cantidad" dataDxfId="17"/>
+    <tableColumn id="3" xr3:uid="{00763216-ACDD-418D-9D9B-0F02D296387E}" name="PrecioUnitario" dataDxfId="16"/>
+    <tableColumn id="4" xr3:uid="{6E6D0715-DC12-452D-8B1E-CF365D12A12B}" name="Porcentaje de descuento" dataDxfId="15"/>
+    <tableColumn id="5" xr3:uid="{B38FD930-D30F-48BA-94A4-68837908CE07}" name="Fecha de envio" dataDxfId="14"/>
+    <tableColumn id="6" xr3:uid="{C066523A-73B4-4BFA-9EA4-BBFD947FE4DC}" name="Comentarios" dataDxfId="13"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -942,13 +942,13 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A1" s="11" t="s">
+      <c r="A1" s="13" t="s">
         <v>11</v>
       </c>
-      <c r="B1" s="11"/>
-      <c r="C1" s="11"/>
-      <c r="D1" s="11"/>
-      <c r="E1" s="11"/>
+      <c r="B1" s="13"/>
+      <c r="C1" s="13"/>
+      <c r="D1" s="13"/>
+      <c r="E1" s="13"/>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
@@ -975,7 +975,7 @@
         <v>14</v>
       </c>
       <c r="C3" s="7" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="D3" s="2">
         <v>46167</v>
@@ -1081,18 +1081,18 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="B1" s="13" t="s">
+      <c r="B1" s="11" t="s">
         <v>21</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A2" s="11" t="s">
+      <c r="A2" s="13" t="s">
         <v>18</v>
       </c>
-      <c r="B2" s="11"/>
-      <c r="C2" s="11"/>
-      <c r="D2" s="11"/>
-      <c r="E2" s="11"/>
+      <c r="B2" s="13"/>
+      <c r="C2" s="13"/>
+      <c r="D2" s="13"/>
+      <c r="E2" s="13"/>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A3" s="8" t="s">
@@ -1113,17 +1113,17 @@
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A4" s="8" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="B4" s="9" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="C4" s="8" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="D4" s="8"/>
       <c r="E4" s="8" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.35">
@@ -1144,14 +1144,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <_activity xmlns="6642a214-a5b4-4988-8240-7802f3742485" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
 <FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
   <Display>DocumentLibraryForm</Display>
@@ -1160,7 +1152,23 @@
 </FormTemplates>
 </file>
 
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <_activity xmlns="6642a214-a5b4-4988-8240-7802f3742485" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<scriptIds xmlns="http://schemas.microsoft.com/office/extensibility/maker/v1.0" id="script-ids-node-id">
+  <scriptId xmlns="" id="ms-officescript%3A%2F%2Fonedrive_business_itemlink%2F01M2JCSHNLA5PAEMN7GBHKBW6MKIKFK2FY:ms-officescript%3A%2F%2Fonedrive_business_sharinglink%2Fu!aHR0cHM6Ly9vbG5hdHVyYS1teS5zaGFyZXBvaW50LmNvbS86dTovcC9iZWNhcmlvX3FyL0lRQ3JCMTRDTWI4d1RxRGJ6RklVVldpNEFlMlUwdlpiaHJBVEd2NWZCUXRYVHln"/>
+  <scriptId xmlns="" id="ms-officescript%3A%2F%2Fonedrive_business_itemlink%2F01M2JCSHNEMVWRZQTUR5HZV776WGJN4BR5:ms-officescript%3A%2F%2Fonedrive_business_sharinglink%2Fu!aHR0cHM6Ly9vbG5hdHVyYS1teS5zaGFyZXBvaW50LmNvbS86dTovcC9iZWNhcmlvX3FyL0lRQ2taVzBjd25TUFQ1cl9fckdTM2dZOUFVbWJCeUJyNFppSXIwZFVYWGhBUENN"/>
+  <scriptId xmlns="" id="ms-officescript%3A%2F%2Fonedrive_business_itemlink%2F01M2JCSHIPJLPFTIZNZFFLYIAQ5ESDY6T3:ms-officescript%3A%2F%2Fonedrive_business_sharinglink%2Fu!aHR0cHM6Ly9vbG5hdHVyYS1teS5zaGFyZXBvaW50LmNvbS86dTovcC9iZWNhcmlvX3FyL0lRQVBTdDVab3kzSlNyd2dFT2trUEhwN0FXZGpxbF9FYmRBbjdROWlaR0h0Y1Nn"/>
+</scriptIds>
+</file>
+
+<file path=customXml/item4.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Documento" ma:contentTypeID="0x01010088D706E71A68E44BB4B903989CF8D857" ma:contentTypeVersion="9" ma:contentTypeDescription="Crear nuevo documento." ma:contentTypeScope="" ma:versionID="7a58337dee26c011ca12ae2bc618b972">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns3="6642a214-a5b4-4988-8240-7802f3742485" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="ddd7c036160bd5eaccfa402a14a53120" ns3:_="">
     <xsd:import namespace="6642a214-a5b4-4988-8240-7802f3742485"/>
@@ -1336,15 +1344,15 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item4.xml><?xml version="1.0" encoding="utf-8"?>
-<scriptIds xmlns="http://schemas.microsoft.com/office/extensibility/maker/v1.0" id="script-ids-node-id">
-  <scriptId xmlns="" id="ms-officescript%3A%2F%2Fonedrive_business_itemlink%2F01M2JCSHNLA5PAEMN7GBHKBW6MKIKFK2FY:ms-officescript%3A%2F%2Fonedrive_business_sharinglink%2Fu!aHR0cHM6Ly9vbG5hdHVyYS1teS5zaGFyZXBvaW50LmNvbS86dTovcC9iZWNhcmlvX3FyL0lRQ3JCMTRDTWI4d1RxRGJ6RklVVldpNEFlMlUwdlpiaHJBVEd2NWZCUXRYVHln"/>
-  <scriptId xmlns="" id="ms-officescript%3A%2F%2Fonedrive_business_itemlink%2F01M2JCSHNEMVWRZQTUR5HZV776WGJN4BR5:ms-officescript%3A%2F%2Fonedrive_business_sharinglink%2Fu!aHR0cHM6Ly9vbG5hdHVyYS1teS5zaGFyZXBvaW50LmNvbS86dTovcC9iZWNhcmlvX3FyL0lRQ2taVzBjd25TUFQ1cl9fckdTM2dZOUFVbWJCeUJyNFppSXIwZFVYWGhBUENN"/>
-  <scriptId xmlns="" id="ms-officescript%3A%2F%2Fonedrive_business_itemlink%2F01M2JCSHIPJLPFTIZNZFFLYIAQ5ESDY6T3:ms-officescript%3A%2F%2Fonedrive_business_sharinglink%2Fu!aHR0cHM6Ly9vbG5hdHVyYS1teS5zaGFyZXBvaW50LmNvbS86dTovcC9iZWNhcmlvX3FyL0lRQVBTdDVab3kzSlNyd2dFT2trUEhwN0FXZGpxbF9FYmRBbjdROWlaR0h0Y1Nn"/>
-</scriptIds>
-</file>
-
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{6BA4C834-A84E-4468-B381-BF97143CCBDE}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{8D1A9822-1768-49DA-A0FE-4E729F91ABFA}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
@@ -1360,15 +1368,16 @@
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{6BA4C834-A84E-4468-B381-BF97143CCBDE}">
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D7178F06-F354-4C81-AF40-EEF0178C64FF}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/extensibility/maker/v1.0"/>
+    <ds:schemaRef ds:uri=""/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps4.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{FE51720D-A8B3-49DF-98E1-66C816B0D7FE}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -1384,13 +1393,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps4.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D7178F06-F354-4C81-AF40-EEF0178C64FF}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/extensibility/maker/v1.0"/>
-    <ds:schemaRef ds:uri=""/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>